<commit_message>
Lisa Eesti finantsstrateegiasse Dalio/Robbins 15–20 mitte-korrelatsioonset voogu
- Uus §2.1 riiklik-kanepiettevotte-mudel.md: Ray Dalio põhimõte ja 18 tuluvoogu
- kanepi-roheline-kuld-raport.md: Eesti Tuleviku Fond + All Seasons viide
- Excel: uus Finantsstrateegia leht mõlemas finantsmudelis

Co-authored-by: reneealuste-commits <reneealuste-commits@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Eesti-Kanepimajandus-5a-Finantsmudel.xlsx
+++ b/Eesti-Kanepimajandus-5a-Finantsmudel.xlsx
@@ -19,6 +19,7 @@
     <sheet name="Brüssel" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="Olemasolevad vahendid" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="Koolid ja loodus" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Finantsstrateegia" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -49,7 +50,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -86,6 +87,11 @@
         <fgColor rgb="001565C0"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="006A1B9A"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -113,7 +119,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -144,6 +150,15 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1514,6 +1529,544 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>EESTI FINANTSSTRATEEGIA — 18 MITTE-KORRELATSIOONSET VOOGU (RAY DALIO / TONY ROBBINS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="11" t="inlineStr">
+        <is>
+          <t>Ray Dalio põhimõte (Tony Robbins *All Seasons*): leia 15–20 mitte-korrelatsioonset tuluvoogu. ERMA kasum → Eesti Tuleviku Fond jaotatakse nii, et üks kriis ei võtab kõike.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>Tuluvoog / varaklass</t>
+        </is>
+      </c>
+      <c r="C4" s="12" t="inlineStr">
+        <is>
+          <t>Korrelatsioon</t>
+        </is>
+      </c>
+      <c r="D4" s="12" t="inlineStr">
+        <is>
+          <t>Siht %</t>
+        </is>
+      </c>
+      <c r="E4" s="12" t="inlineStr">
+        <is>
+          <t>Märkus</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Päikesepargid + salvestus</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Energia ≠ tarbimine</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Macro-kott 40% alamvoog</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Liisingumasinad</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>≠ börs</t>
+        </is>
+      </c>
+      <c r="D6" s="13" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Vaba kassa A5+</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Tööstuskanep eksport</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Ekspordi tsükkel</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Kiud, seemned</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>CBD kosmeetika</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Tarbimine</t>
+        </is>
+      </c>
+      <c r="D8" s="13" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Kreemid, õlid</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Growshop võrgustik</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Kohalik müük</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>25 poodi A5</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Reguleeritud täiskasvanute turg</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Siseriiklik</t>
+        </is>
+      </c>
+      <c r="D10" s="13" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>A3 piloot</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Meditsiiniline kanep</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Haigekassa</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Stabiilne ostja</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Puukoolid + seemik</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Maaelu</t>
+        </is>
+      </c>
+      <c r="D12" s="13" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>30 puukooli</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Kutsekool + koolitus</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Inimkapital</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Uus eriala</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Operation Mirror säästud</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Bürokraatia</t>
+        </is>
+      </c>
+      <c r="D14" s="13" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Koostöö Mirror mudeliga</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>LEADER / EAS / CAP</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Grantid</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>Olemasolev raha</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Urban farm + KOV</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Kogukond</t>
+        </is>
+      </c>
+      <c r="D16" s="13" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Linn + maa</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Teadus + patendid</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Pikaajaline</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>EPM</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Hampcrete + ehitus</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Ehitus</t>
+        </is>
+      </c>
+      <c r="D18" s="13" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>Riigihanke</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Kriisitoit / varud</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Defensiivne</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>2-nädala reegel</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Turism + kogemus</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Hooajaline</t>
+        </is>
+      </c>
+      <c r="D20" s="13" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Farm visits</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>IT + IoT kasvatus</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Tehnoloogia</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>Efektiivsus</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Basic income pilot</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Sotsiaal</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>Macro-kott 20%</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr"/>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>KOKKU</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>18 voogu (Dalio: 15–20)</t>
+        </is>
+      </c>
+      <c r="D23">
+        <f>SUM(D4:D21)</f>
+        <v/>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>100% fondi</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -2229,7 +2782,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2427,7 +2980,11 @@
         <f>F6*0.4</f>
         <v/>
       </c>
-      <c r="G10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Macro-kott</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -2455,7 +3012,11 @@
         <f>F6*0.3</f>
         <v/>
       </c>
-      <c r="G11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Macro-kott</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -2483,7 +3044,11 @@
         <f>F6*0.2</f>
         <v/>
       </c>
-      <c r="G12" t="inlineStr"/>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Macro-kott</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -2511,7 +3076,11 @@
         <f>F6*0.1</f>
         <v/>
       </c>
-      <c r="G13" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Macro-kott</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr"/>
@@ -2525,18 +3094,48 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>5-aasta kumulatiivne EBITDA</t>
-        </is>
-      </c>
-      <c r="B15" s="6">
-        <f>SUM(B6:F6)</f>
-        <v/>
+          <t>Dalio põhimõte</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>18 mitte-korrelatsioonset voogu</t>
+        </is>
       </c>
       <c r="C15" s="6" t="inlineStr"/>
       <c r="D15" s="6" t="inlineStr"/>
       <c r="E15" s="6" t="inlineStr"/>
       <c r="F15" s="6" t="inlineStr"/>
       <c r="G15" t="inlineStr">
+        <is>
+          <t>Vt leht Finantsstrateegia</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr"/>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>5-aasta kumulatiivne EBITDA</t>
+        </is>
+      </c>
+      <c r="B17">
+        <f>SUM(B6:F6)</f>
+        <v/>
+      </c>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
         <is>
           <t>Eesmärk: positiivne A2-st</t>
         </is>

</xml_diff>

<commit_message>
Vähenda finantsstrateegia voogude arv 18 → 8
8 voogu vastavad macro-kottidele 40/30/20/10; Dalio 15–20 jääb viitena.

Co-authored-by: reneealuste-commits <reneealuste-commits@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Eesti-Kanepimajandus-5a-Finantsmudel.xlsx
+++ b/Eesti-Kanepimajandus-5a-Finantsmudel.xlsx
@@ -1535,7 +1535,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1548,14 +1548,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>EESTI FINANTSSTRATEEGIA — 18 MITTE-KORRELATSIOONSET VOOGU (RAY DALIO / TONY ROBBINS)</t>
+          <t>EESTI FINANTSSTRATEEGIA — 8 MITTE-KORRELATSIOONSET VOOGU (RAY DALIO / TONY ROBBINS)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>Ray Dalio põhimõte (Tony Robbins *All Seasons*): leia 15–20 mitte-korrelatsioonset tuluvoogu. ERMA kasum → Eesti Tuleviku Fond jaotatakse nii, et üks kriis ei võtab kõike.</t>
+          <t>Ray Dalio põhimõte (Tony Robbins *All Seasons*): mitte-korrelatsioon (täisversioon 15–20). ERMA kasum → 8 voogu = macro 40/30/20/10.</t>
         </is>
       </c>
     </row>
@@ -1603,11 +1603,11 @@
         </is>
       </c>
       <c r="D5" s="7" t="n">
-        <v>0.12</v>
+        <v>0.4</v>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>Macro-kott 40% alamvoog</t>
+          <t>Macro 40%</t>
         </is>
       </c>
     </row>
@@ -1619,20 +1619,20 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Liisingumasinad</t>
+          <t>Liisingumasinad + robotid</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>≠ börs</t>
+          <t>Tootlik vara ≠ börs</t>
         </is>
       </c>
       <c r="D6" s="13" t="n">
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Vaba kassa A5+</t>
+          <t>Macro 30%</t>
         </is>
       </c>
     </row>
@@ -1644,7 +1644,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Tööstuskanep eksport</t>
+          <t>Tööstuskanep + eksport + CBD</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -1653,11 +1653,11 @@
         </is>
       </c>
       <c r="D7" s="7" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.1</v>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Kiud, seemned</t>
+          <t>Macro 30%</t>
         </is>
       </c>
     </row>
@@ -1669,20 +1669,20 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>CBD kosmeetika</t>
+          <t>Growshop + reguleeritud turg</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Tarbimine</t>
+          <t>Kohalik tarbimine</t>
         </is>
       </c>
       <c r="D8" s="13" t="n">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Kreemid, õlid</t>
+          <t>Macro 30%</t>
         </is>
       </c>
     </row>
@@ -1694,20 +1694,20 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Growshop võrgustik</t>
+          <t>Puukoolid + maaelu (LEADER)</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Kohalik müük</t>
+          <t>Maaelu ≠ börs</t>
         </is>
       </c>
       <c r="D9" s="7" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>25 poodi A5</t>
+          <t>Macro 10%</t>
         </is>
       </c>
     </row>
@@ -1719,12 +1719,12 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Reguleeritud täiskasvanute turg</t>
+          <t>Haridus + kutsekool</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Siseriiklik</t>
+          <t>Inimkapital</t>
         </is>
       </c>
       <c r="D10" s="13" t="n">
@@ -1732,7 +1732,7 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>A3 piloot</t>
+          <t>Macro 10%</t>
         </is>
       </c>
     </row>
@@ -1744,20 +1744,20 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Meditsiiniline kanep</t>
+          <t>Mirror säästud + teadus (EPM)</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Haigekassa</t>
+          <t>Bürokraatia + pikaajaline</t>
         </is>
       </c>
       <c r="D11" s="7" t="n">
-        <v>0.04</v>
+        <v>0.05</v>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Stabiilne ostja</t>
+          <t>Macro 10%</t>
         </is>
       </c>
     </row>
@@ -1769,290 +1769,40 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Puukoolid + seemik</t>
+          <t>Basic income + kriisivarud</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Maaelu</t>
-        </is>
-      </c>
-      <c r="D12" s="13" t="n">
-        <v>0.06</v>
+          <t>Sotsiaal, defensiivne</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>0.2</v>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>30 puukooli</t>
+          <t>Macro 20%</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
+      <c r="A13" s="5" t="inlineStr"/>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Kutsekool + koolitus</t>
+          <t>KOKKU</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Inimkapital</t>
-        </is>
-      </c>
-      <c r="D13" s="7" t="n">
-        <v>0.05</v>
+          <t>8 voogu</t>
+        </is>
+      </c>
+      <c r="D13" s="5">
+        <f>SUM(D4:D11)</f>
+        <v/>
       </c>
       <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>Uus eriala</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>Operation Mirror säästud</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>Bürokraatia</t>
-        </is>
-      </c>
-      <c r="D14" s="13" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="E14" s="3" t="inlineStr">
-        <is>
-          <t>Koostöö Mirror mudeliga</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>LEADER / EAS / CAP</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>Grantid</t>
-        </is>
-      </c>
-      <c r="D15" s="7" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
-          <t>Olemasolev raha</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>Urban farm + KOV</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>Kogukond</t>
-        </is>
-      </c>
-      <c r="D16" s="13" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="E16" s="3" t="inlineStr">
-        <is>
-          <t>Linn + maa</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>Teadus + patendid</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>Pikaajaline</t>
-        </is>
-      </c>
-      <c r="D17" s="7" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="E17" s="5" t="inlineStr">
-        <is>
-          <t>EPM</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>Hampcrete + ehitus</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>Ehitus</t>
-        </is>
-      </c>
-      <c r="D18" s="13" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="E18" s="3" t="inlineStr">
-        <is>
-          <t>Riigihanke</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>Kriisitoit / varud</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>Defensiivne</t>
-        </is>
-      </c>
-      <c r="D19" s="7" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="E19" s="5" t="inlineStr">
-        <is>
-          <t>2-nädala reegel</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>Turism + kogemus</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>Hooajaline</t>
-        </is>
-      </c>
-      <c r="D20" s="13" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="E20" s="3" t="inlineStr">
-        <is>
-          <t>Farm visits</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
-          <t>17</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>IT + IoT kasvatus</t>
-        </is>
-      </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>Tehnoloogia</t>
-        </is>
-      </c>
-      <c r="D21" s="7" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="E21" s="5" t="inlineStr">
-        <is>
-          <t>Efektiivsus</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>Basic income pilot</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>Sotsiaal</t>
-        </is>
-      </c>
-      <c r="D22" s="3" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="E22" s="3" t="inlineStr">
-        <is>
-          <t>Macro-kott 20%</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr"/>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>KOKKU</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>18 voogu (Dalio: 15–20)</t>
-        </is>
-      </c>
-      <c r="D23">
-        <f>SUM(D4:D21)</f>
-        <v/>
-      </c>
-      <c r="E23" t="inlineStr">
         <is>
           <t>100% fondi</t>
         </is>
@@ -2782,7 +2532,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3097,15 +2847,15 @@
           <t>Dalio põhimõte</t>
         </is>
       </c>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>18 mitte-korrelatsioonset voogu</t>
-        </is>
-      </c>
-      <c r="C15" s="6" t="inlineStr"/>
-      <c r="D15" s="6" t="inlineStr"/>
-      <c r="E15" s="6" t="inlineStr"/>
-      <c r="F15" s="6" t="inlineStr"/>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>8 mitte-korrelatsioonset voogu</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr"/>
+      <c r="D15" s="5" t="inlineStr"/>
+      <c r="E15" s="5" t="inlineStr"/>
+      <c r="F15" s="5" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
           <t>Vt leht Finantsstrateegia</t>
@@ -3113,33 +2863,41 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr"/>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
+      <c r="A16" s="3" t="inlineStr"/>
+      <c r="B16" s="3" t="inlineStr"/>
+      <c r="C16" s="3" t="inlineStr"/>
+      <c r="D16" s="3" t="inlineStr"/>
+      <c r="E16" s="3" t="inlineStr"/>
+      <c r="F16" s="3" t="inlineStr"/>
       <c r="G16" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>5-aasta kumulatiivne EBITDA</t>
         </is>
       </c>
-      <c r="B17">
+      <c r="B17" s="5">
         <f>SUM(B6:F6)</f>
         <v/>
       </c>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
+      <c r="C17" s="5" t="inlineStr"/>
+      <c r="D17" s="5" t="inlineStr"/>
+      <c r="E17" s="5" t="inlineStr"/>
+      <c r="F17" s="5" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
           <t>Eesmärk: positiivne A2-st</t>
         </is>
       </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="n"/>
+      <c r="B18" s="4" t="n"/>
+      <c r="C18" s="4" t="n"/>
+      <c r="D18" s="4" t="n"/>
+      <c r="E18" s="4" t="n"/>
+      <c r="F18" s="4" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>